<commit_message>
Update A-Share Blast Lab / 2026-10-26 daily-18:05
</commit_message>
<xml_diff>
--- a/data/theme_strength_latest.xlsx
+++ b/data/theme_strength_latest.xlsx
@@ -218,9 +218,6 @@
     <xf numFmtId="2" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -228,6 +225,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -636,7 +636,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>截至 2026-10-26  2026-10-26 14:55｜每天单独取同类型已合并的题材涨幅前五；日期按降序排列，连续天数截至最新交易日｜板块数据：成分股等权还原（东财板块日线不完整）</t>
+          <t>截至 2026-10-26  2026-10-26 18:11｜每天单独取同类型已合并的题材涨幅前五；日期按降序排列，连续天数截至最新交易日｜板块数据：成分股等权还原（东财板块日线不完整）</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>10-26午盘</t>
+          <t>10-26收盘</t>
         </is>
       </c>
       <c r="L3" s="3" t="n"/>
@@ -973,7 +973,7 @@
       </c>
       <c r="E8" s="12" t="inlineStr"/>
       <c r="F8" s="12" t="n">
-        <v>2.78</v>
+        <v>2.81</v>
       </c>
       <c r="G8" s="12" t="n">
         <v>1</v>
@@ -990,7 +990,7 @@
         </is>
       </c>
       <c r="K8" s="9" t="n">
-        <v>2.78</v>
+        <v>2.81</v>
       </c>
       <c r="L8" s="13" t="n">
         <v>1</v>
@@ -1007,7 +1007,7 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>快递概念</t>
+          <t>可燃冰</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr"/>
       <c r="F9" s="6" t="n">
-        <v>2.08</v>
+        <v>2.15</v>
       </c>
       <c r="G9" s="6" t="n">
         <v>2</v>
@@ -1038,7 +1038,7 @@
         </is>
       </c>
       <c r="K9" s="9" t="n">
-        <v>2.08</v>
+        <v>2.15</v>
       </c>
       <c r="L9" s="10" t="n">
         <v>2</v>
@@ -1055,7 +1055,7 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>乳业</t>
+          <t>快递概念</t>
         </is>
       </c>
       <c r="B10" s="12" t="n">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="E10" s="12" t="inlineStr"/>
       <c r="F10" s="12" t="n">
-        <v>1.96</v>
+        <v>2.11</v>
       </c>
       <c r="G10" s="12" t="n">
         <v>3</v>
@@ -1086,7 +1086,7 @@
         </is>
       </c>
       <c r="K10" s="9" t="n">
-        <v>1.96</v>
+        <v>2.11</v>
       </c>
       <c r="L10" s="13" t="n">
         <v>3</v>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr"/>
       <c r="F11" s="6" t="n">
-        <v>1.94</v>
+        <v>2.01</v>
       </c>
       <c r="G11" s="6" t="n">
         <v>4</v>
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="K11" s="9" t="n">
-        <v>1.94</v>
+        <v>2.01</v>
       </c>
       <c r="L11" s="10" t="n">
         <v>4</v>
@@ -1151,7 +1151,7 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>可燃冰</t>
+          <t>乳业</t>
         </is>
       </c>
       <c r="B12" s="12" t="n">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="E12" s="12" t="inlineStr"/>
       <c r="F12" s="12" t="n">
-        <v>1.89</v>
+        <v>1.99</v>
       </c>
       <c r="G12" s="12" t="n">
         <v>5</v>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="K12" s="9" t="n">
-        <v>1.89</v>
+        <v>1.99</v>
       </c>
       <c r="L12" s="13" t="n">
         <v>5</v>
@@ -1995,7 +1995,7 @@
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>10-26午盘</t>
+          <t>10-26收盘</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="E4" s="16" t="n">
-        <v>2.78</v>
+        <v>2.81</v>
       </c>
       <c r="F4" s="17" t="inlineStr">
         <is>
@@ -2052,10 +2052,10 @@
         <v>7.79</v>
       </c>
       <c r="O4" s="16" t="n">
-        <v>2.83</v>
+        <v>2.78</v>
       </c>
       <c r="P4" s="16" t="n">
-        <v>3.31</v>
+        <v>3.27</v>
       </c>
       <c r="Q4" s="16" t="n">
         <v>1.12</v>
@@ -2068,14 +2068,14 @@
       </c>
       <c r="T4" s="11" t="inlineStr">
         <is>
-          <t>SPD概念 +2.78%</t>
+          <t>SPD概念 +2.81%</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>10-26午盘</t>
+          <t>10-26收盘</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="E5" s="16" t="n">
-        <v>2.78</v>
+        <v>2.81</v>
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
@@ -2132,10 +2132,10 @@
         <v>12.62</v>
       </c>
       <c r="O5" s="16" t="n">
-        <v>7.67</v>
+        <v>7.6</v>
       </c>
       <c r="P5" s="16" t="n">
-        <v>1.64</v>
+        <v>1.62</v>
       </c>
       <c r="Q5" s="16" t="n">
         <v>0.77</v>
@@ -2148,14 +2148,14 @@
       </c>
       <c r="T5" s="11" t="inlineStr">
         <is>
-          <t>SPD概念 +2.78%</t>
+          <t>SPD概念 +2.81%</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>10-26午盘</t>
+          <t>10-26收盘</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
@@ -2172,7 +2172,7 @@
         </is>
       </c>
       <c r="E6" s="16" t="n">
-        <v>2.78</v>
+        <v>2.81</v>
       </c>
       <c r="F6" s="17" t="inlineStr">
         <is>
@@ -2203,519 +2203,519 @@
         </is>
       </c>
       <c r="L6" s="16" t="n">
-        <v>16.83</v>
+        <v>16.8</v>
       </c>
       <c r="M6" s="19" t="n">
-        <v>4.08</v>
+        <v>3.9</v>
       </c>
       <c r="N6" s="19" t="n">
-        <v>0.72</v>
+        <v>0.54</v>
       </c>
       <c r="O6" s="16" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="P6" s="16" t="n">
-        <v>2.03</v>
+        <v>2.06</v>
       </c>
       <c r="Q6" s="16" t="n">
         <v>1.06</v>
       </c>
       <c r="R6" s="16" t="n">
-        <v>-5.66</v>
+        <v>-5.83</v>
       </c>
       <c r="S6" s="16" t="n">
-        <v>13.41</v>
+        <v>13.21</v>
       </c>
       <c r="T6" s="11" t="inlineStr">
         <is>
-          <t>SPD概念 +2.78%</t>
+          <t>SPD概念 +2.81%</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>10-26午盘</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>10-26收盘</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>可燃冰</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>可燃冰</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="F7" s="17" t="inlineStr">
+        <is>
+          <t>领涨前三</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="21" t="inlineStr">
+        <is>
+          <t>601808</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>中海油服</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>油服工程</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>可燃冰、天然气、油气设服、油气资源、海工装备、行业龙头、资源开采概念</t>
+        </is>
+      </c>
+      <c r="L7" s="20" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="M7" s="22" t="n">
+        <v>7.23</v>
+      </c>
+      <c r="N7" s="22" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="O7" s="20" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P7" s="20" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="Q7" s="20" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="R7" s="20" t="n">
+        <v>-33.87</v>
+      </c>
+      <c r="S7" s="20" t="n">
+        <v>25.02</v>
+      </c>
+      <c r="T7" s="5" t="inlineStr">
+        <is>
+          <t>可燃冰 +2.15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>10-26收盘</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>可燃冰</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>可燃冰</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>领涨前三</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="21" t="inlineStr">
+        <is>
+          <t>002278</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>神开股份</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>专用设备</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>可燃冰、无人机、氢能源、碳纤维、页岩气、低空经济、商业航天、油气设服、油气资源、海工装备、长江三角、中俄贸易概念</t>
+        </is>
+      </c>
+      <c r="L8" s="20" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="M8" s="22" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="N8" s="22" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="O8" s="20" t="n">
+        <v>8.58</v>
+      </c>
+      <c r="P8" s="20" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="Q8" s="20" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="R8" s="20" t="n">
+        <v>-50.06</v>
+      </c>
+      <c r="S8" s="20" t="n">
+        <v>10.03</v>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>可燃冰 +2.15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="38" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>10-26收盘</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>可燃冰</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>可燃冰</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="F9" s="17" t="inlineStr">
+        <is>
+          <t>领涨前三</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" s="21" t="inlineStr">
+        <is>
+          <t>000039</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>中集集团</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>通用设备</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>风能、可燃冰、天然气、氢能源、物联网、冷链物流、商业航天、数据中心、油气资源、海工装备、深圳特区、社保新进、雄安新区</t>
+        </is>
+      </c>
+      <c r="L9" s="20" t="n">
+        <v>8.609999999999999</v>
+      </c>
+      <c r="M9" s="22" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="N9" s="22" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="O9" s="20" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="P9" s="20" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="Q9" s="20" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="R9" s="20" t="n">
+        <v>-36.32</v>
+      </c>
+      <c r="S9" s="20" t="n">
+        <v>18.27</v>
+      </c>
+      <c r="T9" s="5" t="inlineStr">
+        <is>
+          <t>可燃冰 +2.15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="38" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>10-26收盘</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>快递概念</t>
         </is>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C10" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>快递概念</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>领涨前三</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>001317</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>三羊马</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>铁路公路</t>
+        </is>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>快递概念、跨境电商、统一大市场、西部大开发</t>
+        </is>
+      </c>
+      <c r="L10" s="16" t="n">
+        <v>53.68</v>
+      </c>
+      <c r="M10" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="N10" s="23" t="n">
+        <v>-1.86</v>
+      </c>
+      <c r="O10" s="16" t="n">
+        <v>14.05</v>
+      </c>
+      <c r="P10" s="16" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="Q10" s="16" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="R10" s="16" t="n">
+        <v>-21.36</v>
+      </c>
+      <c r="S10" s="16" t="n">
+        <v>37.61</v>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>快递概念 +2.11%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="38" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>10-26收盘</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>快递概念</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>快递概念</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="F11" s="17" t="inlineStr">
+        <is>
+          <t>领涨前三</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="H11" s="18" t="inlineStr">
+        <is>
+          <t>002468</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>申通快递</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr">
+        <is>
+          <t>物流</t>
+        </is>
+      </c>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>大数据、小盘价值、快递概念、阿里概念</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="n">
+        <v>14.68</v>
+      </c>
+      <c r="M11" s="19" t="n">
+        <v>5.84</v>
+      </c>
+      <c r="N11" s="19" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="O11" s="16" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="P11" s="16" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="Q11" s="16" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="R11" s="16" t="n">
+        <v>-18.13</v>
+      </c>
+      <c r="S11" s="16" t="n">
+        <v>17.63</v>
+      </c>
+      <c r="T11" s="11" t="inlineStr">
+        <is>
+          <t>快递概念 +2.11%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="38" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>10-26收盘</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>快递概念</t>
         </is>
       </c>
-      <c r="E7" s="16" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="F7" s="17" t="inlineStr">
+      <c r="C12" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>快递概念</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
         <is>
           <t>领涨前三</t>
         </is>
       </c>
-      <c r="G7" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="18" t="inlineStr">
-        <is>
-          <t>001317</t>
-        </is>
-      </c>
-      <c r="I7" s="11" t="inlineStr">
-        <is>
-          <t>三羊马</t>
-        </is>
-      </c>
-      <c r="J7" s="11" t="inlineStr">
-        <is>
-          <t>铁路公路</t>
-        </is>
-      </c>
-      <c r="K7" s="11" t="inlineStr">
-        <is>
-          <t>快递概念、跨境电商、统一大市场、西部大开发</t>
-        </is>
-      </c>
-      <c r="L7" s="16" t="n">
-        <v>53.68</v>
-      </c>
-      <c r="M7" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="N7" s="20" t="n">
-        <v>-1.86</v>
-      </c>
-      <c r="O7" s="16" t="n">
-        <v>14.17</v>
-      </c>
-      <c r="P7" s="16" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="Q7" s="16" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="R7" s="16" t="n">
-        <v>-21.36</v>
-      </c>
-      <c r="S7" s="16" t="n">
-        <v>37.61</v>
-      </c>
-      <c r="T7" s="11" t="inlineStr">
-        <is>
-          <t>快递概念 +2.08%</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>10-26午盘</t>
-        </is>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>快递概念</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>快递概念</t>
-        </is>
-      </c>
-      <c r="E8" s="16" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="F8" s="17" t="inlineStr">
-        <is>
-          <t>领涨前三</t>
-        </is>
-      </c>
-      <c r="G8" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="H8" s="18" t="inlineStr">
-        <is>
-          <t>002468</t>
-        </is>
-      </c>
-      <c r="I8" s="11" t="inlineStr">
-        <is>
-          <t>申通快递</t>
-        </is>
-      </c>
-      <c r="J8" s="11" t="inlineStr">
+      <c r="G12" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>601598</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>中国外运</t>
+        </is>
+      </c>
+      <c r="J12" s="11" t="inlineStr">
         <is>
           <t>物流</t>
         </is>
       </c>
-      <c r="K8" s="11" t="inlineStr">
-        <is>
-          <t>大数据、小盘价值、快递概念、阿里概念</t>
-        </is>
-      </c>
-      <c r="L8" s="16" t="n">
-        <v>14.7</v>
-      </c>
-      <c r="M8" s="19" t="n">
-        <v>5.98</v>
-      </c>
-      <c r="N8" s="19" t="n">
-        <v>1.73</v>
-      </c>
-      <c r="O8" s="16" t="n">
-        <v>1.82</v>
-      </c>
-      <c r="P8" s="16" t="n">
-        <v>1.76</v>
-      </c>
-      <c r="Q8" s="16" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="R8" s="16" t="n">
-        <v>-18.01</v>
-      </c>
-      <c r="S8" s="16" t="n">
-        <v>17.79</v>
-      </c>
-      <c r="T8" s="11" t="inlineStr">
-        <is>
-          <t>快递概念 +2.08%</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="38" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>10-26午盘</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>快递概念</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D9" s="11" t="inlineStr">
-        <is>
-          <t>快递概念</t>
-        </is>
-      </c>
-      <c r="E9" s="16" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="F9" s="17" t="inlineStr">
-        <is>
-          <t>领涨前三</t>
-        </is>
-      </c>
-      <c r="G9" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="H9" s="18" t="inlineStr">
-        <is>
-          <t>601598</t>
-        </is>
-      </c>
-      <c r="I9" s="11" t="inlineStr">
-        <is>
-          <t>中国外运</t>
-        </is>
-      </c>
-      <c r="J9" s="11" t="inlineStr">
-        <is>
-          <t>物流</t>
-        </is>
-      </c>
-      <c r="K9" s="11" t="inlineStr">
+      <c r="K12" s="11" t="inlineStr">
         <is>
           <t>中盘价值、冷链物流、快递概念、跨境电商、统一大市场</t>
         </is>
       </c>
-      <c r="L9" s="16" t="n">
-        <v>6.79</v>
-      </c>
-      <c r="M9" s="19" t="n">
-        <v>5.11</v>
-      </c>
-      <c r="N9" s="20" t="n">
-        <v>-1.45</v>
-      </c>
-      <c r="O9" s="16" t="n">
+      <c r="L12" s="16" t="n">
+        <v>6.81</v>
+      </c>
+      <c r="M12" s="19" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="N12" s="23" t="n">
+        <v>-1.16</v>
+      </c>
+      <c r="O12" s="16" t="n">
         <v>0.36</v>
       </c>
-      <c r="P9" s="16" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="Q9" s="16" t="n">
+      <c r="P12" s="16" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="Q12" s="16" t="n">
         <v>0.87</v>
       </c>
-      <c r="R9" s="16" t="n">
-        <v>-2.02</v>
-      </c>
-      <c r="S9" s="16" t="n">
-        <v>36.9</v>
-      </c>
-      <c r="T9" s="11" t="inlineStr">
-        <is>
-          <t>快递概念 +2.08%</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="38" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>10-26午盘</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>乳业</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>乳业</t>
-        </is>
-      </c>
-      <c r="E10" s="21" t="n">
-        <v>1.96</v>
-      </c>
-      <c r="F10" s="17" t="inlineStr">
-        <is>
-          <t>领涨前三</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="22" t="inlineStr">
-        <is>
-          <t>001219</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>青岛食品</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>休闲食品</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>乳业、婴童概念、电商概念、网红经济、调味品概念</t>
-        </is>
-      </c>
-      <c r="L10" s="21" t="n">
-        <v>13.62</v>
-      </c>
-      <c r="M10" s="23" t="n">
-        <v>10.02</v>
-      </c>
-      <c r="N10" s="23" t="n">
-        <v>9.66</v>
-      </c>
-      <c r="O10" s="21" t="n">
-        <v>4.02</v>
-      </c>
-      <c r="P10" s="21" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="Q10" s="21" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="R10" s="21" t="n">
-        <v>-12.36</v>
-      </c>
-      <c r="S10" s="21" t="n">
-        <v>18.85</v>
-      </c>
-      <c r="T10" s="5" t="inlineStr">
-        <is>
-          <t>乳业 +1.96%</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="38" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>10-26午盘</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>乳业</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>乳业</t>
-        </is>
-      </c>
-      <c r="E11" s="21" t="n">
-        <v>1.96</v>
-      </c>
-      <c r="F11" s="17" t="inlineStr">
-        <is>
-          <t>领涨前三</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="H11" s="22" t="inlineStr">
-        <is>
-          <t>001318</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>阳光乳业</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>饮料乳品</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>乳业、味蕾经济、婴童概念</t>
-        </is>
-      </c>
-      <c r="L11" s="21" t="n">
-        <v>12.1</v>
-      </c>
-      <c r="M11" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="N11" s="24" t="n">
-        <v>-11.94</v>
-      </c>
-      <c r="O11" s="21" t="n">
-        <v>13.58</v>
-      </c>
-      <c r="P11" s="21" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="Q11" s="21" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="R11" s="21" t="n">
-        <v>-30.22</v>
-      </c>
-      <c r="S11" s="21" t="n">
-        <v>26.57</v>
-      </c>
-      <c r="T11" s="5" t="inlineStr">
-        <is>
-          <t>乳业 +1.96%</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="38" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>10-26午盘</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>乳业</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>乳业</t>
-        </is>
-      </c>
-      <c r="E12" s="21" t="n">
-        <v>1.96</v>
-      </c>
-      <c r="F12" s="17" t="inlineStr">
-        <is>
-          <t>领涨前三</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H12" s="22" t="inlineStr">
-        <is>
-          <t>603719</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>良品铺子</t>
-        </is>
-      </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>休闲食品</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>乳业、内贸流通、电商概念、社区团购、网红经济、谷子经济</t>
-        </is>
-      </c>
-      <c r="L12" s="21" t="n">
-        <v>9.390000000000001</v>
-      </c>
-      <c r="M12" s="23" t="n">
-        <v>9.949999999999999</v>
-      </c>
-      <c r="N12" s="23" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="O12" s="21" t="n">
-        <v>3.46</v>
-      </c>
-      <c r="P12" s="21" t="n">
-        <v>3.51</v>
-      </c>
-      <c r="Q12" s="21" t="n">
-        <v>1.43</v>
-      </c>
-      <c r="R12" s="21" t="n">
-        <v>-26.35</v>
-      </c>
-      <c r="S12" s="21" t="n">
-        <v>14.65</v>
-      </c>
-      <c r="T12" s="5" t="inlineStr">
-        <is>
-          <t>乳业 +1.96%</t>
+      <c r="R12" s="16" t="n">
+        <v>-1.73</v>
+      </c>
+      <c r="S12" s="16" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="T12" s="11" t="inlineStr">
+        <is>
+          <t>快递概念 +2.11%</t>
         </is>
       </c>
     </row>
     <row r="13" ht="38" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>10-26午盘</t>
+          <t>10-26收盘</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -2731,8 +2731,8 @@
           <t>电子竞技</t>
         </is>
       </c>
-      <c r="E13" s="21" t="n">
-        <v>1.94</v>
+      <c r="E13" s="20" t="n">
+        <v>2.01</v>
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
@@ -2742,7 +2742,7 @@
       <c r="G13" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="22" t="inlineStr">
+      <c r="H13" s="21" t="inlineStr">
         <is>
           <t>603258</t>
         </is>
@@ -2762,40 +2762,40 @@
           <t>文娱消费、电子竞技、网络游戏、虚拟现实、谷子经济、AIGC概念、短剧互动游戏</t>
         </is>
       </c>
-      <c r="L13" s="21" t="n">
+      <c r="L13" s="20" t="n">
         <v>15.3</v>
       </c>
-      <c r="M13" s="23" t="n">
+      <c r="M13" s="22" t="n">
         <v>9.99</v>
       </c>
-      <c r="N13" s="23" t="n">
+      <c r="N13" s="22" t="n">
         <v>4.37</v>
       </c>
-      <c r="O13" s="21" t="n">
-        <v>7.59</v>
-      </c>
-      <c r="P13" s="21" t="n">
-        <v>1.52</v>
-      </c>
-      <c r="Q13" s="21" t="n">
+      <c r="O13" s="20" t="n">
+        <v>7.46</v>
+      </c>
+      <c r="P13" s="20" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q13" s="20" t="n">
         <v>1.18</v>
       </c>
-      <c r="R13" s="21" t="n">
+      <c r="R13" s="20" t="n">
         <v>-26.02</v>
       </c>
-      <c r="S13" s="21" t="n">
+      <c r="S13" s="20" t="n">
         <v>41.4</v>
       </c>
       <c r="T13" s="5" t="inlineStr">
         <is>
-          <t>电子竞技 +1.94%</t>
+          <t>电子竞技 +2.01%</t>
         </is>
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>10-26午盘</t>
+          <t>10-26收盘</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -2811,8 +2811,8 @@
           <t>电子竞技</t>
         </is>
       </c>
-      <c r="E14" s="21" t="n">
-        <v>1.94</v>
+      <c r="E14" s="20" t="n">
+        <v>2.01</v>
       </c>
       <c r="F14" s="17" t="inlineStr">
         <is>
@@ -2822,7 +2822,7 @@
       <c r="G14" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H14" s="22" t="inlineStr">
+      <c r="H14" s="21" t="inlineStr">
         <is>
           <t>001308</t>
         </is>
@@ -2842,40 +2842,40 @@
           <t>AIPC、AI眼镜、OLED、华为概念、小盘价值、智能电视、智能穿戴、深圳特区、电子竞技、虚拟现实、贬值受益、医疗器械概念、消费电子概念、MiniLED、抖音概念(字节概念)</t>
         </is>
       </c>
-      <c r="L14" s="21" t="n">
-        <v>19.15</v>
-      </c>
-      <c r="M14" s="23" t="n">
-        <v>3.46</v>
-      </c>
-      <c r="N14" s="23" t="n">
-        <v>6.98</v>
-      </c>
-      <c r="O14" s="21" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="P14" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q14" s="21" t="n">
+      <c r="L14" s="20" t="n">
+        <v>19.17</v>
+      </c>
+      <c r="M14" s="22" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="N14" s="22" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="O14" s="20" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="P14" s="20" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="Q14" s="20" t="n">
         <v>1.47</v>
       </c>
-      <c r="R14" s="21" t="n">
-        <v>-12.91</v>
-      </c>
-      <c r="S14" s="21" t="n">
-        <v>17.7</v>
+      <c r="R14" s="20" t="n">
+        <v>-12.82</v>
+      </c>
+      <c r="S14" s="20" t="n">
+        <v>17.82</v>
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>电子竞技 +1.94%</t>
+          <t>电子竞技 +2.01%</t>
         </is>
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>10-26午盘</t>
+          <t>10-26收盘</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -2891,8 +2891,8 @@
           <t>电子竞技</t>
         </is>
       </c>
-      <c r="E15" s="21" t="n">
-        <v>1.94</v>
+      <c r="E15" s="20" t="n">
+        <v>2.01</v>
       </c>
       <c r="F15" s="17" t="inlineStr">
         <is>
@@ -2902,7 +2902,7 @@
       <c r="G15" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H15" s="22" t="inlineStr">
+      <c r="H15" s="21" t="inlineStr">
         <is>
           <t>002517</t>
         </is>
@@ -2922,45 +2922,45 @@
           <t>AI眼镜、华为概念、文娱消费、电子竞技、网络游戏、虚拟现实、短剧互动游戏</t>
         </is>
       </c>
-      <c r="L15" s="21" t="n">
-        <v>15.55</v>
-      </c>
-      <c r="M15" s="23" t="n">
-        <v>3.32</v>
-      </c>
-      <c r="N15" s="23" t="n">
-        <v>1.97</v>
-      </c>
-      <c r="O15" s="21" t="n">
-        <v>2.41</v>
-      </c>
-      <c r="P15" s="21" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="Q15" s="21" t="n">
+      <c r="L15" s="20" t="n">
+        <v>15.57</v>
+      </c>
+      <c r="M15" s="22" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="N15" s="22" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="O15" s="20" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="P15" s="20" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="Q15" s="20" t="n">
         <v>1.03</v>
       </c>
-      <c r="R15" s="21" t="n">
-        <v>-43.27</v>
-      </c>
-      <c r="S15" s="21" t="n">
-        <v>9.66</v>
+      <c r="R15" s="20" t="n">
+        <v>-43.2</v>
+      </c>
+      <c r="S15" s="20" t="n">
+        <v>9.800000000000001</v>
       </c>
       <c r="T15" s="5" t="inlineStr">
         <is>
-          <t>电子竞技 +1.94%</t>
+          <t>电子竞技 +2.01%</t>
         </is>
       </c>
     </row>
     <row r="16" ht="38" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>10-26午盘</t>
+          <t>10-26收盘</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>可燃冰</t>
+          <t>乳业</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
@@ -2968,11 +2968,11 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>可燃冰</t>
-        </is>
-      </c>
-      <c r="E16" s="21" t="n">
-        <v>1.89</v>
+          <t>乳业</t>
+        </is>
+      </c>
+      <c r="E16" s="20" t="n">
+        <v>1.99</v>
       </c>
       <c r="F16" s="17" t="inlineStr">
         <is>
@@ -2982,65 +2982,65 @@
       <c r="G16" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H16" s="22" t="inlineStr">
-        <is>
-          <t>601808</t>
+      <c r="H16" s="21" t="inlineStr">
+        <is>
+          <t>001219</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>中海油服</t>
+          <t>青岛食品</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>油服工程</t>
+          <t>休闲食品</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>可燃冰、天然气、油气设服、油气资源、海工装备、行业龙头、资源开采概念</t>
-        </is>
-      </c>
-      <c r="L16" s="21" t="n">
-        <v>13.47</v>
-      </c>
-      <c r="M16" s="23" t="n">
-        <v>7.07</v>
-      </c>
-      <c r="N16" s="23" t="n">
-        <v>4.66</v>
-      </c>
-      <c r="O16" s="21" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="P16" s="21" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="Q16" s="21" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="R16" s="21" t="n">
-        <v>-33.97</v>
-      </c>
-      <c r="S16" s="21" t="n">
-        <v>24.84</v>
+          <t>乳业、婴童概念、电商概念、网红经济、调味品概念</t>
+        </is>
+      </c>
+      <c r="L16" s="20" t="n">
+        <v>13.62</v>
+      </c>
+      <c r="M16" s="22" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="N16" s="22" t="n">
+        <v>9.66</v>
+      </c>
+      <c r="O16" s="20" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="P16" s="20" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="Q16" s="20" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="R16" s="20" t="n">
+        <v>-12.36</v>
+      </c>
+      <c r="S16" s="20" t="n">
+        <v>18.85</v>
       </c>
       <c r="T16" s="5" t="inlineStr">
         <is>
-          <t>可燃冰 +1.89%</t>
+          <t>乳业 +1.99%</t>
         </is>
       </c>
     </row>
     <row r="17" ht="38" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>10-26午盘</t>
+          <t>10-26收盘</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>可燃冰</t>
+          <t>乳业</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
@@ -3048,11 +3048,11 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>可燃冰</t>
-        </is>
-      </c>
-      <c r="E17" s="21" t="n">
-        <v>1.89</v>
+          <t>乳业</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="n">
+        <v>1.99</v>
       </c>
       <c r="F17" s="17" t="inlineStr">
         <is>
@@ -3062,65 +3062,65 @@
       <c r="G17" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H17" s="22" t="inlineStr">
-        <is>
-          <t>002278</t>
+      <c r="H17" s="21" t="inlineStr">
+        <is>
+          <t>001318</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>神开股份</t>
+          <t>阳光乳业</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>专用设备</t>
+          <t>饮料乳品</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>可燃冰、无人机、氢能源、碳纤维、页岩气、低空经济、商业航天、油气设服、油气资源、海工装备、长江三角、中俄贸易概念</t>
-        </is>
-      </c>
-      <c r="L17" s="21" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="M17" s="23" t="n">
-        <v>3.67</v>
-      </c>
-      <c r="N17" s="23" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="O17" s="21" t="n">
-        <v>8.57</v>
-      </c>
-      <c r="P17" s="21" t="n">
-        <v>2.13</v>
-      </c>
-      <c r="Q17" s="21" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="R17" s="21" t="n">
-        <v>-50.06</v>
-      </c>
-      <c r="S17" s="21" t="n">
-        <v>10.03</v>
+          <t>乳业、味蕾经济、婴童概念</t>
+        </is>
+      </c>
+      <c r="L17" s="20" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="M17" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="N17" s="24" t="n">
+        <v>-11.94</v>
+      </c>
+      <c r="O17" s="20" t="n">
+        <v>13.32</v>
+      </c>
+      <c r="P17" s="20" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="Q17" s="20" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="R17" s="20" t="n">
+        <v>-30.22</v>
+      </c>
+      <c r="S17" s="20" t="n">
+        <v>26.57</v>
       </c>
       <c r="T17" s="5" t="inlineStr">
         <is>
-          <t>可燃冰 +1.89%</t>
+          <t>乳业 +1.99%</t>
         </is>
       </c>
     </row>
     <row r="18" ht="38" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>10-26午盘</t>
+          <t>10-26收盘</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>可燃冰</t>
+          <t>乳业</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
@@ -3128,11 +3128,11 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>可燃冰</t>
-        </is>
-      </c>
-      <c r="E18" s="21" t="n">
-        <v>1.89</v>
+          <t>乳业</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="n">
+        <v>1.99</v>
       </c>
       <c r="F18" s="17" t="inlineStr">
         <is>
@@ -3142,53 +3142,53 @@
       <c r="G18" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H18" s="22" t="inlineStr">
-        <is>
-          <t>000039</t>
+      <c r="H18" s="21" t="inlineStr">
+        <is>
+          <t>603719</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>中集集团</t>
+          <t>良品铺子</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>通用设备</t>
+          <t>休闲食品</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>风能、可燃冰、天然气、氢能源、物联网、冷链物流、商业航天、数据中心、油气资源、海工装备、深圳特区、社保新进、雄安新区</t>
-        </is>
-      </c>
-      <c r="L18" s="21" t="n">
-        <v>8.59</v>
-      </c>
-      <c r="M18" s="23" t="n">
-        <v>2.63</v>
-      </c>
-      <c r="N18" s="23" t="n">
-        <v>7.37</v>
-      </c>
-      <c r="O18" s="21" t="n">
-        <v>1.87</v>
-      </c>
-      <c r="P18" s="21" t="n">
-        <v>1.64</v>
-      </c>
-      <c r="Q18" s="21" t="n">
-        <v>1.19</v>
-      </c>
-      <c r="R18" s="21" t="n">
-        <v>-36.46</v>
-      </c>
-      <c r="S18" s="21" t="n">
-        <v>17.99</v>
+          <t>乳业、内贸流通、电商概念、社区团购、网红经济、谷子经济</t>
+        </is>
+      </c>
+      <c r="L18" s="20" t="n">
+        <v>9.390000000000001</v>
+      </c>
+      <c r="M18" s="22" t="n">
+        <v>9.949999999999999</v>
+      </c>
+      <c r="N18" s="22" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="O18" s="20" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="P18" s="20" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="Q18" s="20" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="R18" s="20" t="n">
+        <v>-26.35</v>
+      </c>
+      <c r="S18" s="20" t="n">
+        <v>14.65</v>
       </c>
       <c r="T18" s="5" t="inlineStr">
         <is>
-          <t>可燃冰 +1.89%</t>
+          <t>乳业 +1.99%</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4411,7 @@
           <t>虚拟机器人</t>
         </is>
       </c>
-      <c r="E34" s="21" t="n">
+      <c r="E34" s="20" t="n">
         <v>5.59</v>
       </c>
       <c r="F34" s="17" t="inlineStr">
@@ -4422,7 +4422,7 @@
       <c r="G34" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H34" s="22" t="inlineStr">
+      <c r="H34" s="21" t="inlineStr">
         <is>
           <t>603528</t>
         </is>
@@ -4442,28 +4442,28 @@
           <t>大数据、物联网、华为昇腾、华为概念、卫星导航、国产芯片、国产软件、智慧城市、职业教育、虚拟机器人、车联网(车路云)</t>
         </is>
       </c>
-      <c r="L34" s="21" t="n">
+      <c r="L34" s="20" t="n">
         <v>8.140000000000001</v>
       </c>
-      <c r="M34" s="23" t="n">
+      <c r="M34" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="N34" s="23" t="n">
+      <c r="N34" s="22" t="n">
         <v>24.66</v>
       </c>
-      <c r="O34" s="21" t="n">
+      <c r="O34" s="20" t="n">
         <v>12.51</v>
       </c>
-      <c r="P34" s="21" t="n">
+      <c r="P34" s="20" t="n">
         <v>3.14</v>
       </c>
-      <c r="Q34" s="21" t="n">
+      <c r="Q34" s="20" t="n">
         <v>1.6</v>
       </c>
-      <c r="R34" s="21" t="n">
+      <c r="R34" s="20" t="n">
         <v>-28.47</v>
       </c>
-      <c r="S34" s="21" t="n">
+      <c r="S34" s="20" t="n">
         <v>49.91</v>
       </c>
       <c r="T34" s="5" t="inlineStr">
@@ -4491,7 +4491,7 @@
           <t>虚拟机器人</t>
         </is>
       </c>
-      <c r="E35" s="21" t="n">
+      <c r="E35" s="20" t="n">
         <v>5.59</v>
       </c>
       <c r="F35" s="17" t="inlineStr">
@@ -4502,7 +4502,7 @@
       <c r="G35" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H35" s="22" t="inlineStr">
+      <c r="H35" s="21" t="inlineStr">
         <is>
           <t>601519</t>
         </is>
@@ -4522,28 +4522,28 @@
           <t>大数据、华为概念、国产软件、小盘成长、数据中心、私募重仓、网红经济、长江三角、阿里概念、高市净率、鸿蒙概念、互联网金融、虚拟机器人</t>
         </is>
       </c>
-      <c r="L35" s="21" t="n">
+      <c r="L35" s="20" t="n">
         <v>9.25</v>
       </c>
-      <c r="M35" s="23" t="n">
+      <c r="M35" s="22" t="n">
         <v>9.99</v>
       </c>
       <c r="N35" s="24" t="n">
         <v>-2.43</v>
       </c>
-      <c r="O35" s="21" t="n">
+      <c r="O35" s="20" t="n">
         <v>6.2</v>
       </c>
-      <c r="P35" s="21" t="n">
+      <c r="P35" s="20" t="n">
         <v>1.54</v>
       </c>
-      <c r="Q35" s="21" t="n">
+      <c r="Q35" s="20" t="n">
         <v>1.02</v>
       </c>
-      <c r="R35" s="21" t="n">
+      <c r="R35" s="20" t="n">
         <v>-39.62</v>
       </c>
-      <c r="S35" s="21" t="n">
+      <c r="S35" s="20" t="n">
         <v>24.33</v>
       </c>
       <c r="T35" s="5" t="inlineStr">
@@ -4571,7 +4571,7 @@
           <t>虚拟机器人</t>
         </is>
       </c>
-      <c r="E36" s="21" t="n">
+      <c r="E36" s="20" t="n">
         <v>5.59</v>
       </c>
       <c r="F36" s="17" t="inlineStr">
@@ -4582,7 +4582,7 @@
       <c r="G36" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H36" s="22" t="inlineStr">
+      <c r="H36" s="21" t="inlineStr">
         <is>
           <t>001314</t>
         </is>
@@ -4602,28 +4602,28 @@
           <t>PCB、物联网、AIPC、AI眼镜、在线教育、增强现实、智能穿戴、虚拟现实、虚拟机器人、消费电子概念</t>
         </is>
       </c>
-      <c r="L36" s="21" t="n">
+      <c r="L36" s="20" t="n">
         <v>45.33</v>
       </c>
-      <c r="M36" s="23" t="n">
+      <c r="M36" s="22" t="n">
         <v>5.62</v>
       </c>
-      <c r="N36" s="23" t="n">
+      <c r="N36" s="22" t="n">
         <v>6.66</v>
       </c>
-      <c r="O36" s="21" t="n">
+      <c r="O36" s="20" t="n">
         <v>4.67</v>
       </c>
-      <c r="P36" s="21" t="n">
+      <c r="P36" s="20" t="n">
         <v>1.66</v>
       </c>
-      <c r="Q36" s="21" t="n">
+      <c r="Q36" s="20" t="n">
         <v>1.09</v>
       </c>
-      <c r="R36" s="21" t="n">
+      <c r="R36" s="20" t="n">
         <v>-29.48</v>
       </c>
-      <c r="S36" s="21" t="n">
+      <c r="S36" s="20" t="n">
         <v>18.05</v>
       </c>
       <c r="T36" s="5" t="inlineStr">
@@ -4688,7 +4688,7 @@
       <c r="M37" s="19" t="n">
         <v>3.85</v>
       </c>
-      <c r="N37" s="20" t="n">
+      <c r="N37" s="23" t="n">
         <v>-0.53</v>
       </c>
       <c r="O37" s="16" t="n">
@@ -4765,10 +4765,10 @@
       <c r="L38" s="16" t="n">
         <v>14.3</v>
       </c>
-      <c r="M38" s="20" t="n">
+      <c r="M38" s="23" t="n">
         <v>-4.41</v>
       </c>
-      <c r="N38" s="20" t="n">
+      <c r="N38" s="23" t="n">
         <v>-6.9</v>
       </c>
       <c r="O38" s="16" t="n">
@@ -4811,7 +4811,7 @@
           <t>ChatGPT概念</t>
         </is>
       </c>
-      <c r="E39" s="21" t="n">
+      <c r="E39" s="20" t="n">
         <v>5.2</v>
       </c>
       <c r="F39" s="17" t="inlineStr">
@@ -4822,7 +4822,7 @@
       <c r="G39" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H39" s="22" t="inlineStr">
+      <c r="H39" s="21" t="inlineStr">
         <is>
           <t>603466</t>
         </is>
@@ -4842,28 +4842,28 @@
           <t>全息技术、华为概念、数字孪生、旅游概念、百度概念、网红经济、网络游戏、职业教育、脑机接口、虚拟现实、裸眼3D、超清视频、首发经济、新型城镇化、虚拟数字人、AIGC概念、ChatGPT概念、DeepSeek概念</t>
         </is>
       </c>
-      <c r="L39" s="21" t="n">
+      <c r="L39" s="20" t="n">
         <v>14.69</v>
       </c>
-      <c r="M39" s="23" t="n">
+      <c r="M39" s="22" t="n">
         <v>10.04</v>
       </c>
-      <c r="N39" s="23" t="n">
+      <c r="N39" s="22" t="n">
         <v>16.22</v>
       </c>
-      <c r="O39" s="21" t="n">
+      <c r="O39" s="20" t="n">
         <v>16.7</v>
       </c>
-      <c r="P39" s="21" t="n">
+      <c r="P39" s="20" t="n">
         <v>1.29</v>
       </c>
-      <c r="Q39" s="21" t="n">
+      <c r="Q39" s="20" t="n">
         <v>1.47</v>
       </c>
-      <c r="R39" s="21" t="n">
+      <c r="R39" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="S39" s="21" t="n">
+      <c r="S39" s="20" t="n">
         <v>66.36</v>
       </c>
       <c r="T39" s="5" t="inlineStr">
@@ -4891,7 +4891,7 @@
           <t>ChatGPT概念</t>
         </is>
       </c>
-      <c r="E40" s="21" t="n">
+      <c r="E40" s="20" t="n">
         <v>5.2</v>
       </c>
       <c r="F40" s="17" t="inlineStr">
@@ -4902,7 +4902,7 @@
       <c r="G40" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H40" s="22" t="inlineStr">
+      <c r="H40" s="21" t="inlineStr">
         <is>
           <t>002354</t>
         </is>
@@ -4922,28 +4922,28 @@
           <t>信创、AI语料、东数西算、国产芯片、在线教育、小盘价值、文娱消费、电子竞技、百度概念、网络游戏、股权分散、虚拟现实、谷子经济、跨境电商、互联网服务、互联网金融、多模态AI、小红书概念、虚拟数字人、AIGC概念、Web3.0、短剧互动游戏、ChatGPT概念、DeepSeek概念、抖音概念(字节概念)</t>
         </is>
       </c>
-      <c r="L40" s="21" t="n">
+      <c r="L40" s="20" t="n">
         <v>8.029999999999999</v>
       </c>
-      <c r="M40" s="23" t="n">
+      <c r="M40" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="N40" s="23" t="n">
+      <c r="N40" s="22" t="n">
         <v>11.37</v>
       </c>
-      <c r="O40" s="21" t="n">
+      <c r="O40" s="20" t="n">
         <v>17.93</v>
       </c>
-      <c r="P40" s="21" t="n">
+      <c r="P40" s="20" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q40" s="21" t="n">
+      <c r="Q40" s="20" t="n">
         <v>1.25</v>
       </c>
-      <c r="R40" s="21" t="n">
+      <c r="R40" s="20" t="n">
         <v>-22.34</v>
       </c>
-      <c r="S40" s="21" t="n">
+      <c r="S40" s="20" t="n">
         <v>48.43</v>
       </c>
       <c r="T40" s="5" t="inlineStr">
@@ -4971,7 +4971,7 @@
           <t>ChatGPT概念</t>
         </is>
       </c>
-      <c r="E41" s="21" t="n">
+      <c r="E41" s="20" t="n">
         <v>5.2</v>
       </c>
       <c r="F41" s="17" t="inlineStr">
@@ -4982,7 +4982,7 @@
       <c r="G41" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H41" s="22" t="inlineStr">
+      <c r="H41" s="21" t="inlineStr">
         <is>
           <t>600446</t>
         </is>
@@ -5002,28 +5002,28 @@
           <t>信创、国产软件、数据安全、智慧城市、深圳特区、电商概念、网络安全、股权分散、互联网服务、虚拟机器人、ChatGPT概念</t>
         </is>
       </c>
-      <c r="L41" s="21" t="n">
+      <c r="L41" s="20" t="n">
         <v>10.6</v>
       </c>
-      <c r="M41" s="23" t="n">
+      <c r="M41" s="22" t="n">
         <v>5.37</v>
       </c>
-      <c r="N41" s="23" t="n">
+      <c r="N41" s="22" t="n">
         <v>3.01</v>
       </c>
-      <c r="O41" s="21" t="n">
+      <c r="O41" s="20" t="n">
         <v>3.2</v>
       </c>
-      <c r="P41" s="21" t="n">
+      <c r="P41" s="20" t="n">
         <v>2.06</v>
       </c>
-      <c r="Q41" s="21" t="n">
+      <c r="Q41" s="20" t="n">
         <v>1.14</v>
       </c>
-      <c r="R41" s="21" t="n">
+      <c r="R41" s="20" t="n">
         <v>-40.62</v>
       </c>
-      <c r="S41" s="21" t="n">
+      <c r="S41" s="20" t="n">
         <v>8.720000000000001</v>
       </c>
       <c r="T41" s="5" t="inlineStr">
@@ -5485,7 +5485,7 @@
       <c r="L47" s="16" t="n">
         <v>7.29</v>
       </c>
-      <c r="M47" s="20" t="n">
+      <c r="M47" s="23" t="n">
         <v>-1.62</v>
       </c>
       <c r="N47" s="19" t="n">
@@ -5691,7 +5691,7 @@
           <t>轮毂电机</t>
         </is>
       </c>
-      <c r="E50" s="21" t="n">
+      <c r="E50" s="20" t="n">
         <v>0.16</v>
       </c>
       <c r="F50" s="17" t="inlineStr">
@@ -5702,7 +5702,7 @@
       <c r="G50" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H50" s="22" t="inlineStr">
+      <c r="H50" s="21" t="inlineStr">
         <is>
           <t>603350</t>
         </is>
@@ -5722,28 +5722,28 @@
           <t>传感器、轮毂电机</t>
         </is>
       </c>
-      <c r="L50" s="21" t="n">
+      <c r="L50" s="20" t="n">
         <v>29.48</v>
       </c>
-      <c r="M50" s="23" t="n">
+      <c r="M50" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="N50" s="23" t="n">
+      <c r="N50" s="22" t="n">
         <v>12.01</v>
       </c>
-      <c r="O50" s="21" t="n">
+      <c r="O50" s="20" t="n">
         <v>5.79</v>
       </c>
-      <c r="P50" s="21" t="n">
+      <c r="P50" s="20" t="n">
         <v>4.23</v>
       </c>
-      <c r="Q50" s="21" t="n">
+      <c r="Q50" s="20" t="n">
         <v>1.55</v>
       </c>
-      <c r="R50" s="21" t="n">
+      <c r="R50" s="20" t="n">
         <v>-27.28</v>
       </c>
-      <c r="S50" s="21" t="n">
+      <c r="S50" s="20" t="n">
         <v>13.65</v>
       </c>
       <c r="T50" s="5" t="inlineStr">
@@ -5771,7 +5771,7 @@
           <t>轮毂电机</t>
         </is>
       </c>
-      <c r="E51" s="21" t="n">
+      <c r="E51" s="20" t="n">
         <v>0.16</v>
       </c>
       <c r="F51" s="17" t="inlineStr">
@@ -5782,7 +5782,7 @@
       <c r="G51" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H51" s="22" t="inlineStr">
+      <c r="H51" s="21" t="inlineStr">
         <is>
           <t>603489</t>
         </is>
@@ -5802,28 +5802,28 @@
           <t>交运设备、共享经济、轮毂电机</t>
         </is>
       </c>
-      <c r="L51" s="21" t="n">
+      <c r="L51" s="20" t="n">
         <v>27.5</v>
       </c>
-      <c r="M51" s="23" t="n">
+      <c r="M51" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="N51" s="23" t="n">
+      <c r="N51" s="22" t="n">
         <v>6.51</v>
       </c>
-      <c r="O51" s="21" t="n">
+      <c r="O51" s="20" t="n">
         <v>1.31</v>
       </c>
-      <c r="P51" s="21" t="n">
+      <c r="P51" s="20" t="n">
         <v>1.46</v>
       </c>
-      <c r="Q51" s="21" t="n">
+      <c r="Q51" s="20" t="n">
         <v>1.06</v>
       </c>
-      <c r="R51" s="21" t="n">
+      <c r="R51" s="20" t="n">
         <v>-31.13</v>
       </c>
-      <c r="S51" s="21" t="n">
+      <c r="S51" s="20" t="n">
         <v>16.48</v>
       </c>
       <c r="T51" s="5" t="inlineStr">
@@ -5851,7 +5851,7 @@
           <t>轮毂电机</t>
         </is>
       </c>
-      <c r="E52" s="21" t="n">
+      <c r="E52" s="20" t="n">
         <v>0.16</v>
       </c>
       <c r="F52" s="17" t="inlineStr">
@@ -5862,7 +5862,7 @@
       <c r="G52" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H52" s="22" t="inlineStr">
+      <c r="H52" s="21" t="inlineStr">
         <is>
           <t>002284</t>
         </is>
@@ -5882,28 +5882,28 @@
           <t>华为汽车、胎压监测、轮毂电机、长江三角、车联网(车路云)</t>
         </is>
       </c>
-      <c r="L52" s="21" t="n">
+      <c r="L52" s="20" t="n">
         <v>8.57</v>
       </c>
       <c r="M52" s="24" t="n">
         <v>-0.58</v>
       </c>
-      <c r="N52" s="23" t="n">
+      <c r="N52" s="22" t="n">
         <v>3.38</v>
       </c>
-      <c r="O52" s="21" t="n">
+      <c r="O52" s="20" t="n">
         <v>1.2</v>
       </c>
-      <c r="P52" s="21" t="n">
+      <c r="P52" s="20" t="n">
         <v>0.64</v>
       </c>
-      <c r="Q52" s="21" t="n">
+      <c r="Q52" s="20" t="n">
         <v>0.77</v>
       </c>
-      <c r="R52" s="21" t="n">
+      <c r="R52" s="20" t="n">
         <v>-50.58</v>
       </c>
-      <c r="S52" s="21" t="n">
+      <c r="S52" s="20" t="n">
         <v>3.38</v>
       </c>
       <c r="T52" s="5" t="inlineStr">
@@ -6205,7 +6205,7 @@
       <c r="L56" s="16" t="n">
         <v>13.27</v>
       </c>
-      <c r="M56" s="20" t="n">
+      <c r="M56" s="23" t="n">
         <v>-9.970000000000001</v>
       </c>
       <c r="N56" s="19" t="n">
@@ -6525,7 +6525,7 @@
       <c r="L60" s="16" t="n">
         <v>7.29</v>
       </c>
-      <c r="M60" s="20" t="n">
+      <c r="M60" s="23" t="n">
         <v>-1.62</v>
       </c>
       <c r="N60" s="19" t="n">
@@ -7005,7 +7005,7 @@
       <c r="L66" s="16" t="n">
         <v>10.61</v>
       </c>
-      <c r="M66" s="20" t="n">
+      <c r="M66" s="23" t="n">
         <v>-0.47</v>
       </c>
       <c r="N66" s="19" t="n">
@@ -7248,7 +7248,7 @@
       <c r="M69" s="19" t="n">
         <v>1.51</v>
       </c>
-      <c r="N69" s="20" t="n">
+      <c r="N69" s="23" t="n">
         <v>-2.44</v>
       </c>
       <c r="O69" s="16" t="n">
@@ -7291,7 +7291,7 @@
           <t>知识产权</t>
         </is>
       </c>
-      <c r="E70" s="21" t="n">
+      <c r="E70" s="20" t="n">
         <v>2.34</v>
       </c>
       <c r="F70" s="17" t="inlineStr">
@@ -7302,7 +7302,7 @@
       <c r="G70" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H70" s="22" t="inlineStr">
+      <c r="H70" s="21" t="inlineStr">
         <is>
           <t>603999</t>
         </is>
@@ -7322,28 +7322,28 @@
           <t>快手概念、知识产权、西部大开发</t>
         </is>
       </c>
-      <c r="L70" s="21" t="n">
+      <c r="L70" s="20" t="n">
         <v>7.47</v>
       </c>
-      <c r="M70" s="23" t="n">
+      <c r="M70" s="22" t="n">
         <v>10.01</v>
       </c>
-      <c r="N70" s="23" t="n">
+      <c r="N70" s="22" t="n">
         <v>7.79</v>
       </c>
-      <c r="O70" s="21" t="n">
+      <c r="O70" s="20" t="n">
         <v>11.65</v>
       </c>
-      <c r="P70" s="21" t="n">
+      <c r="P70" s="20" t="n">
         <v>2.42</v>
       </c>
-      <c r="Q70" s="21" t="n">
+      <c r="Q70" s="20" t="n">
         <v>1.55</v>
       </c>
-      <c r="R70" s="21" t="n">
+      <c r="R70" s="20" t="n">
         <v>-15.21</v>
       </c>
-      <c r="S70" s="21" t="n">
+      <c r="S70" s="20" t="n">
         <v>51.21</v>
       </c>
       <c r="T70" s="5" t="inlineStr">
@@ -7371,7 +7371,7 @@
           <t>知识产权</t>
         </is>
       </c>
-      <c r="E71" s="21" t="n">
+      <c r="E71" s="20" t="n">
         <v>2.34</v>
       </c>
       <c r="F71" s="17" t="inlineStr">
@@ -7382,7 +7382,7 @@
       <c r="G71" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H71" s="22" t="inlineStr">
+      <c r="H71" s="21" t="inlineStr">
         <is>
           <t>601999</t>
         </is>
@@ -7402,28 +7402,28 @@
           <t>东北振兴、在线教育、基金减仓、知识产权</t>
         </is>
       </c>
-      <c r="L71" s="21" t="n">
+      <c r="L71" s="20" t="n">
         <v>7.8</v>
       </c>
-      <c r="M71" s="23" t="n">
+      <c r="M71" s="22" t="n">
         <v>10.01</v>
       </c>
-      <c r="N71" s="23" t="n">
+      <c r="N71" s="22" t="n">
         <v>6.7</v>
       </c>
-      <c r="O71" s="21" t="n">
+      <c r="O71" s="20" t="n">
         <v>3.24</v>
       </c>
-      <c r="P71" s="21" t="n">
+      <c r="P71" s="20" t="n">
         <v>0.53</v>
       </c>
-      <c r="Q71" s="21" t="n">
+      <c r="Q71" s="20" t="n">
         <v>1.23</v>
       </c>
-      <c r="R71" s="21" t="n">
+      <c r="R71" s="20" t="n">
         <v>-7.14</v>
       </c>
-      <c r="S71" s="21" t="n">
+      <c r="S71" s="20" t="n">
         <v>44.44</v>
       </c>
       <c r="T71" s="5" t="inlineStr">
@@ -7451,7 +7451,7 @@
           <t>知识产权</t>
         </is>
       </c>
-      <c r="E72" s="21" t="n">
+      <c r="E72" s="20" t="n">
         <v>2.34</v>
       </c>
       <c r="F72" s="17" t="inlineStr">
@@ -7462,7 +7462,7 @@
       <c r="G72" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H72" s="22" t="inlineStr">
+      <c r="H72" s="21" t="inlineStr">
         <is>
           <t>603721</t>
         </is>
@@ -7482,28 +7482,28 @@
           <t>AI语料、体育产业、影视概念、数字水印、文娱消费、旅游概念、知识产权、网红经济、职业教育、虚拟现实、超清视频、小红书概念、短剧互动游戏</t>
         </is>
       </c>
-      <c r="L72" s="21" t="n">
+      <c r="L72" s="20" t="n">
         <v>20.82</v>
       </c>
-      <c r="M72" s="23" t="n">
+      <c r="M72" s="22" t="n">
         <v>9.98</v>
       </c>
-      <c r="N72" s="23" t="n">
+      <c r="N72" s="22" t="n">
         <v>3.22</v>
       </c>
-      <c r="O72" s="21" t="n">
+      <c r="O72" s="20" t="n">
         <v>9.44</v>
       </c>
-      <c r="P72" s="21" t="n">
+      <c r="P72" s="20" t="n">
         <v>1.37</v>
       </c>
-      <c r="Q72" s="21" t="n">
+      <c r="Q72" s="20" t="n">
         <v>1.18</v>
       </c>
-      <c r="R72" s="21" t="n">
+      <c r="R72" s="20" t="n">
         <v>-19.49</v>
       </c>
-      <c r="S72" s="21" t="n">
+      <c r="S72" s="20" t="n">
         <v>44.58</v>
       </c>
       <c r="T72" s="5" t="inlineStr">
@@ -7648,7 +7648,7 @@
       <c r="M74" s="19" t="n">
         <v>2.9</v>
       </c>
-      <c r="N74" s="20" t="n">
+      <c r="N74" s="23" t="n">
         <v>-0.93</v>
       </c>
       <c r="O74" s="16" t="n">
@@ -8125,7 +8125,7 @@
       <c r="L80" s="16" t="n">
         <v>11.75</v>
       </c>
-      <c r="M80" s="20" t="n">
+      <c r="M80" s="23" t="n">
         <v>-6.52</v>
       </c>
       <c r="N80" s="19" t="n">
@@ -8571,7 +8571,7 @@
           <t>WiFi</t>
         </is>
       </c>
-      <c r="E86" s="21" t="n">
+      <c r="E86" s="20" t="n">
         <v>4.02</v>
       </c>
       <c r="F86" s="17" t="inlineStr">
@@ -8582,7 +8582,7 @@
       <c r="G86" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H86" s="22" t="inlineStr">
+      <c r="H86" s="21" t="inlineStr">
         <is>
           <t>603068</t>
         </is>
@@ -8602,28 +8602,28 @@
           <t>ETC、无人机、物联网、AI眼镜、WiFi、华为概念、卫星导航、国产芯片、小米概念、无线耳机、汽车芯片、算力概念、通信技术、阿里概念、半导体概念、消费电子概念</t>
         </is>
       </c>
-      <c r="L86" s="21" t="n">
+      <c r="L86" s="20" t="n">
         <v>41.67</v>
       </c>
-      <c r="M86" s="23" t="n">
+      <c r="M86" s="22" t="n">
         <v>10.01</v>
       </c>
-      <c r="N86" s="23" t="n">
+      <c r="N86" s="22" t="n">
         <v>1.51</v>
       </c>
-      <c r="O86" s="21" t="n">
+      <c r="O86" s="20" t="n">
         <v>8.279999999999999</v>
       </c>
-      <c r="P86" s="21" t="n">
+      <c r="P86" s="20" t="n">
         <v>0.83</v>
       </c>
-      <c r="Q86" s="21" t="n">
+      <c r="Q86" s="20" t="n">
         <v>0.83</v>
       </c>
-      <c r="R86" s="21" t="n">
+      <c r="R86" s="20" t="n">
         <v>-14.1</v>
       </c>
-      <c r="S86" s="21" t="n">
+      <c r="S86" s="20" t="n">
         <v>37.52</v>
       </c>
       <c r="T86" s="5" t="inlineStr">
@@ -8651,7 +8651,7 @@
           <t>WiFi</t>
         </is>
       </c>
-      <c r="E87" s="21" t="n">
+      <c r="E87" s="20" t="n">
         <v>4.02</v>
       </c>
       <c r="F87" s="17" t="inlineStr">
@@ -8662,7 +8662,7 @@
       <c r="G87" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H87" s="22" t="inlineStr">
+      <c r="H87" s="21" t="inlineStr">
         <is>
           <t>001388</t>
         </is>
@@ -8682,28 +8682,28 @@
           <t>PCB、物联网、特高压、5G概念、WiFi、国产软件、基金减仓、智能电网、机器视觉、激光雷达、算力概念、通信技术、多模态AI、工业互联网、新型工业化、电子身份证、中俄贸易概念</t>
         </is>
       </c>
-      <c r="L87" s="21" t="n">
+      <c r="L87" s="20" t="n">
         <v>20.37</v>
       </c>
-      <c r="M87" s="23" t="n">
+      <c r="M87" s="22" t="n">
         <v>9.99</v>
       </c>
-      <c r="N87" s="23" t="n">
+      <c r="N87" s="22" t="n">
         <v>3.56</v>
       </c>
-      <c r="O87" s="21" t="n">
+      <c r="O87" s="20" t="n">
         <v>8.44</v>
       </c>
-      <c r="P87" s="21" t="n">
+      <c r="P87" s="20" t="n">
         <v>2.7</v>
       </c>
-      <c r="Q87" s="21" t="n">
+      <c r="Q87" s="20" t="n">
         <v>0.97</v>
       </c>
-      <c r="R87" s="21" t="n">
+      <c r="R87" s="20" t="n">
         <v>-36.9</v>
       </c>
-      <c r="S87" s="21" t="n">
+      <c r="S87" s="20" t="n">
         <v>19.75</v>
       </c>
       <c r="T87" s="5" t="inlineStr">
@@ -8731,7 +8731,7 @@
           <t>WiFi</t>
         </is>
       </c>
-      <c r="E88" s="21" t="n">
+      <c r="E88" s="20" t="n">
         <v>4.02</v>
       </c>
       <c r="F88" s="17" t="inlineStr">
@@ -8742,7 +8742,7 @@
       <c r="G88" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H88" s="22" t="inlineStr">
+      <c r="H88" s="21" t="inlineStr">
         <is>
           <t>002792</t>
         </is>
@@ -8762,28 +8762,28 @@
           <t>5G概念、6G概念、WiFi、低空经济、储能概念、卫星导航、商业航天、通信技术、F5G概念、UWB概念、光通信模块、卫星互联网、毫米波概念、中俄贸易概念</t>
         </is>
       </c>
-      <c r="L88" s="21" t="n">
+      <c r="L88" s="20" t="n">
         <v>29.17</v>
       </c>
-      <c r="M88" s="23" t="n">
+      <c r="M88" s="22" t="n">
         <v>9.289999999999999</v>
       </c>
-      <c r="N88" s="23" t="n">
+      <c r="N88" s="22" t="n">
         <v>6.3</v>
       </c>
-      <c r="O88" s="21" t="n">
+      <c r="O88" s="20" t="n">
         <v>12.75</v>
       </c>
-      <c r="P88" s="21" t="n">
+      <c r="P88" s="20" t="n">
         <v>1.66</v>
       </c>
-      <c r="Q88" s="21" t="n">
+      <c r="Q88" s="20" t="n">
         <v>0.79</v>
       </c>
-      <c r="R88" s="21" t="n">
+      <c r="R88" s="20" t="n">
         <v>-58.3</v>
       </c>
-      <c r="S88" s="21" t="n">
+      <c r="S88" s="20" t="n">
         <v>70.78</v>
       </c>
       <c r="T88" s="5" t="inlineStr">
@@ -8848,7 +8848,7 @@
       <c r="M89" s="19" t="n">
         <v>0.57</v>
       </c>
-      <c r="N89" s="20" t="n">
+      <c r="N89" s="23" t="n">
         <v>-3.7</v>
       </c>
       <c r="O89" s="16" t="n">
@@ -8925,10 +8925,10 @@
       <c r="L90" s="16" t="n">
         <v>15.63</v>
       </c>
-      <c r="M90" s="20" t="n">
+      <c r="M90" s="23" t="n">
         <v>-0.13</v>
       </c>
-      <c r="N90" s="20" t="n">
+      <c r="N90" s="23" t="n">
         <v>-3.28</v>
       </c>
       <c r="O90" s="16" t="n">
@@ -8971,7 +8971,7 @@
           <t>AI芯片</t>
         </is>
       </c>
-      <c r="E91" s="21" t="n">
+      <c r="E91" s="20" t="n">
         <v>3.86</v>
       </c>
       <c r="F91" s="17" t="inlineStr">
@@ -8982,7 +8982,7 @@
       <c r="G91" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H91" s="22" t="inlineStr">
+      <c r="H91" s="21" t="inlineStr">
         <is>
           <t>603893</t>
         </is>
@@ -9002,28 +9002,28 @@
           <t>物联网、AI眼镜、AI芯片、华为概念、国产芯片、大盘成长、百度概念、虚拟现实、高市净率、EDR概念、半导体概念</t>
         </is>
       </c>
-      <c r="L91" s="21" t="n">
+      <c r="L91" s="20" t="n">
         <v>189.04</v>
       </c>
-      <c r="M91" s="23" t="n">
+      <c r="M91" s="22" t="n">
         <v>10</v>
       </c>
       <c r="N91" s="24" t="n">
         <v>-3.84</v>
       </c>
-      <c r="O91" s="21" t="n">
+      <c r="O91" s="20" t="n">
         <v>4.96</v>
       </c>
-      <c r="P91" s="21" t="n">
+      <c r="P91" s="20" t="n">
         <v>1.57</v>
       </c>
-      <c r="Q91" s="21" t="n">
+      <c r="Q91" s="20" t="n">
         <v>1.17</v>
       </c>
-      <c r="R91" s="21" t="n">
+      <c r="R91" s="20" t="n">
         <v>-16.96</v>
       </c>
-      <c r="S91" s="21" t="n">
+      <c r="S91" s="20" t="n">
         <v>30.62</v>
       </c>
       <c r="T91" s="5" t="inlineStr">
@@ -9051,7 +9051,7 @@
           <t>AI芯片</t>
         </is>
       </c>
-      <c r="E92" s="21" t="n">
+      <c r="E92" s="20" t="n">
         <v>3.86</v>
       </c>
       <c r="F92" s="17" t="inlineStr">
@@ -9062,7 +9062,7 @@
       <c r="G92" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H92" s="22" t="inlineStr">
+      <c r="H92" s="21" t="inlineStr">
         <is>
           <t>002195</t>
         </is>
@@ -9082,28 +9082,28 @@
           <t>大数据、AIPC、AI芯片、AI语料、中盘成长、华为概念、国产软件、百度概念、网络安全、网络游戏、股权分散、脑机接口、长江三角、阿里概念、首发经济、鸿蒙概念、互联网服务、互联网金融、多模态AI、AIGC概念、短剧互动游戏、AI制药（医疗）、抖音概念(字节概念)</t>
         </is>
       </c>
-      <c r="L92" s="21" t="n">
+      <c r="L92" s="20" t="n">
         <v>5.88</v>
       </c>
-      <c r="M92" s="23" t="n">
+      <c r="M92" s="22" t="n">
         <v>2.62</v>
       </c>
       <c r="N92" s="24" t="n">
         <v>-2.49</v>
       </c>
-      <c r="O92" s="21" t="n">
+      <c r="O92" s="20" t="n">
         <v>1.79</v>
       </c>
-      <c r="P92" s="21" t="n">
+      <c r="P92" s="20" t="n">
         <v>1.32</v>
       </c>
-      <c r="Q92" s="21" t="n">
+      <c r="Q92" s="20" t="n">
         <v>1.12</v>
       </c>
-      <c r="R92" s="21" t="n">
+      <c r="R92" s="20" t="n">
         <v>-55.42</v>
       </c>
-      <c r="S92" s="21" t="n">
+      <c r="S92" s="20" t="n">
         <v>2.8</v>
       </c>
       <c r="T92" s="5" t="inlineStr">
@@ -9131,7 +9131,7 @@
           <t>AI芯片</t>
         </is>
       </c>
-      <c r="E93" s="21" t="n">
+      <c r="E93" s="20" t="n">
         <v>3.86</v>
       </c>
       <c r="F93" s="17" t="inlineStr">
@@ -9142,7 +9142,7 @@
       <c r="G93" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H93" s="22" t="inlineStr">
+      <c r="H93" s="21" t="inlineStr">
         <is>
           <t>002049</t>
         </is>
@@ -9162,28 +9162,28 @@
           <t>军工、ETC、大飞机、碳化硅、蓝宝石、5G概念、AI芯片、商业航天、国产芯片、存储芯片、汽车芯片、算力概念、通信技术、半导体概念、卫星互联网、高带宽内存、IGBT概念、车联网(车路云)</t>
         </is>
       </c>
-      <c r="L93" s="21" t="n">
+      <c r="L93" s="20" t="n">
         <v>53.97</v>
       </c>
-      <c r="M93" s="23" t="n">
+      <c r="M93" s="22" t="n">
         <v>2.6</v>
       </c>
       <c r="N93" s="24" t="n">
         <v>-2.55</v>
       </c>
-      <c r="O93" s="21" t="n">
+      <c r="O93" s="20" t="n">
         <v>1.24</v>
       </c>
-      <c r="P93" s="21" t="n">
+      <c r="P93" s="20" t="n">
         <v>1.1</v>
       </c>
-      <c r="Q93" s="21" t="n">
+      <c r="Q93" s="20" t="n">
         <v>1.03</v>
       </c>
-      <c r="R93" s="21" t="n">
+      <c r="R93" s="20" t="n">
         <v>-41.64</v>
       </c>
-      <c r="S93" s="21" t="n">
+      <c r="S93" s="20" t="n">
         <v>3.49</v>
       </c>
       <c r="T93" s="5" t="inlineStr">
@@ -9485,7 +9485,7 @@
       <c r="L97" s="16" t="n">
         <v>28.18</v>
       </c>
-      <c r="M97" s="20" t="n">
+      <c r="M97" s="23" t="n">
         <v>-1.88</v>
       </c>
       <c r="N97" s="19" t="n">
@@ -9885,7 +9885,7 @@
       <c r="L102" s="16" t="n">
         <v>15.77</v>
       </c>
-      <c r="M102" s="20" t="n">
+      <c r="M102" s="23" t="n">
         <v>-0.88</v>
       </c>
       <c r="N102" s="19" t="n">

</xml_diff>

<commit_message>
Update A-Share Blast Lab / 2026-10-27 close-update-retry2
</commit_message>
<xml_diff>
--- a/data/theme_strength_latest.xlsx
+++ b/data/theme_strength_latest.xlsx
@@ -650,7 +650,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>截至 2026-10-27  2026-10-27 14:55｜每天单独取同类型已合并的题材涨幅前五；日期按降序排列，连续天数截至最新交易日｜板块数据：成分股等权还原（东财板块日线不完整）</t>
+          <t>截至 2026-10-27  2026-10-27 18:10｜每天单独取同类型已合并的题材涨幅前五；日期按降序排列，连续天数截至最新交易日｜板块数据：成分股等权还原（东财板块日线不完整）</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="L3" s="3" t="n"/>
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.83</v>
+        <v>0.77</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>4.5</v>
@@ -840,7 +840,7 @@
         </is>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-0.15</v>
+        <v>-0.26</v>
       </c>
       <c r="L5" s="8" t="n">
         <v>4</v>
@@ -987,7 +987,7 @@
       </c>
       <c r="E8" s="13" t="inlineStr"/>
       <c r="F8" s="13" t="n">
-        <v>1.32</v>
+        <v>1.3</v>
       </c>
       <c r="G8" s="13" t="n">
         <v>1.5</v>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="K8" s="9" t="n">
-        <v>2.48</v>
+        <v>2.43</v>
       </c>
       <c r="L8" s="14" t="n">
         <v>1</v>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="E9" s="16" t="inlineStr"/>
       <c r="F9" s="16" t="n">
-        <v>1.05</v>
+        <v>0.99</v>
       </c>
       <c r="G9" s="16" t="n">
         <v>2</v>
@@ -1056,7 +1056,7 @@
         </is>
       </c>
       <c r="K9" s="9" t="n">
-        <v>1.05</v>
+        <v>0.99</v>
       </c>
       <c r="L9" s="17" t="n">
         <v>2</v>
@@ -1087,7 +1087,7 @@
       </c>
       <c r="E10" s="13" t="inlineStr"/>
       <c r="F10" s="13" t="n">
-        <v>0.27</v>
+        <v>0.13</v>
       </c>
       <c r="G10" s="13" t="n">
         <v>3</v>
@@ -1104,7 +1104,7 @@
         </is>
       </c>
       <c r="K10" s="9" t="n">
-        <v>0.27</v>
+        <v>0.13</v>
       </c>
       <c r="L10" s="14" t="n">
         <v>3</v>
@@ -1135,7 +1135,7 @@
       </c>
       <c r="E11" s="16" t="inlineStr"/>
       <c r="F11" s="16" t="n">
-        <v>-0.39</v>
+        <v>-0.47</v>
       </c>
       <c r="G11" s="16" t="n">
         <v>5</v>
@@ -1152,7 +1152,7 @@
         </is>
       </c>
       <c r="K11" s="7" t="n">
-        <v>-0.39</v>
+        <v>-0.47</v>
       </c>
       <c r="L11" s="17" t="n">
         <v>5</v>
@@ -2013,7 +2013,7 @@
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B4" s="12" t="inlineStr">
@@ -2030,7 +2030,7 @@
         </is>
       </c>
       <c r="E4" s="19" t="n">
-        <v>2.48</v>
+        <v>2.43</v>
       </c>
       <c r="F4" s="20" t="inlineStr">
         <is>
@@ -2070,10 +2070,10 @@
         <v>10.51</v>
       </c>
       <c r="O4" s="19" t="n">
-        <v>6.81</v>
+        <v>6.79</v>
       </c>
       <c r="P4" s="19" t="n">
-        <v>3.44</v>
+        <v>3.43</v>
       </c>
       <c r="Q4" s="19" t="n">
         <v>1.34</v>
@@ -2086,14 +2086,14 @@
       </c>
       <c r="T4" s="12" t="inlineStr">
         <is>
-          <t>轮毂电机 +2.48%</t>
+          <t>轮毂电机 +2.43%</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
@@ -2110,7 +2110,7 @@
         </is>
       </c>
       <c r="E5" s="19" t="n">
-        <v>2.48</v>
+        <v>2.43</v>
       </c>
       <c r="F5" s="20" t="inlineStr">
         <is>
@@ -2141,39 +2141,39 @@
         </is>
       </c>
       <c r="L5" s="19" t="n">
-        <v>29.93</v>
+        <v>29.9</v>
       </c>
       <c r="M5" s="22" t="n">
-        <v>9.390000000000001</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="N5" s="22" t="n">
-        <v>9.07</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="O5" s="19" t="n">
-        <v>3.85</v>
+        <v>3.92</v>
       </c>
       <c r="P5" s="19" t="n">
-        <v>3.67</v>
+        <v>3.72</v>
       </c>
       <c r="Q5" s="19" t="n">
         <v>1.6</v>
       </c>
       <c r="R5" s="19" t="n">
-        <v>-25.04</v>
+        <v>-25.12</v>
       </c>
       <c r="S5" s="19" t="n">
-        <v>26.77</v>
+        <v>26.64</v>
       </c>
       <c r="T5" s="12" t="inlineStr">
         <is>
-          <t>轮毂电机 +2.48%</t>
+          <t>轮毂电机 +2.43%</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="E6" s="19" t="n">
-        <v>2.48</v>
+        <v>2.43</v>
       </c>
       <c r="F6" s="20" t="inlineStr">
         <is>
@@ -2221,39 +2221,39 @@
         </is>
       </c>
       <c r="L6" s="19" t="n">
-        <v>30.13</v>
+        <v>30.17</v>
       </c>
       <c r="M6" s="22" t="n">
-        <v>5.94</v>
+        <v>6.08</v>
       </c>
       <c r="N6" s="22" t="n">
-        <v>10.85</v>
+        <v>11</v>
       </c>
       <c r="O6" s="19" t="n">
-        <v>15.01</v>
+        <v>15.15</v>
       </c>
       <c r="P6" s="19" t="n">
-        <v>4.4</v>
+        <v>4.43</v>
       </c>
       <c r="Q6" s="19" t="n">
         <v>2.96</v>
       </c>
       <c r="R6" s="19" t="n">
-        <v>-25.68</v>
+        <v>-25.58</v>
       </c>
       <c r="S6" s="19" t="n">
-        <v>16.15</v>
+        <v>16.31</v>
       </c>
       <c r="T6" s="12" t="inlineStr">
         <is>
-          <t>轮毂电机 +2.48%</t>
+          <t>轮毂电机 +2.43%</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
@@ -2270,7 +2270,7 @@
         </is>
       </c>
       <c r="E7" s="19" t="n">
-        <v>2.48</v>
+        <v>2.43</v>
       </c>
       <c r="F7" s="23" t="inlineStr">
         <is>
@@ -2301,39 +2301,39 @@
         </is>
       </c>
       <c r="L7" s="19" t="n">
-        <v>10.12</v>
+        <v>10.1</v>
       </c>
       <c r="M7" s="22" t="n">
-        <v>5.75</v>
+        <v>5.54</v>
       </c>
       <c r="N7" s="22" t="n">
-        <v>4.01</v>
+        <v>3.8</v>
       </c>
       <c r="O7" s="19" t="n">
-        <v>6.34</v>
+        <v>6.39</v>
       </c>
       <c r="P7" s="19" t="n">
-        <v>4.52</v>
+        <v>4.54</v>
       </c>
       <c r="Q7" s="19" t="n">
         <v>1.65</v>
       </c>
       <c r="R7" s="19" t="n">
-        <v>-37.22</v>
+        <v>-37.34</v>
       </c>
       <c r="S7" s="19" t="n">
-        <v>18.22</v>
+        <v>17.99</v>
       </c>
       <c r="T7" s="12" t="inlineStr">
         <is>
-          <t>轮毂电机 +2.48%</t>
+          <t>轮毂电机 +2.43%</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B8" s="12" t="inlineStr">
@@ -2350,7 +2350,7 @@
         </is>
       </c>
       <c r="E8" s="19" t="n">
-        <v>2.48</v>
+        <v>2.43</v>
       </c>
       <c r="F8" s="23" t="inlineStr">
         <is>
@@ -2381,39 +2381,39 @@
         </is>
       </c>
       <c r="L8" s="19" t="n">
-        <v>30.13</v>
+        <v>30.17</v>
       </c>
       <c r="M8" s="22" t="n">
-        <v>5.94</v>
+        <v>6.08</v>
       </c>
       <c r="N8" s="22" t="n">
-        <v>10.85</v>
+        <v>11</v>
       </c>
       <c r="O8" s="19" t="n">
-        <v>15.01</v>
+        <v>15.15</v>
       </c>
       <c r="P8" s="19" t="n">
-        <v>4.4</v>
+        <v>4.43</v>
       </c>
       <c r="Q8" s="19" t="n">
         <v>2.96</v>
       </c>
       <c r="R8" s="19" t="n">
-        <v>-25.68</v>
+        <v>-25.58</v>
       </c>
       <c r="S8" s="19" t="n">
-        <v>16.15</v>
+        <v>16.31</v>
       </c>
       <c r="T8" s="12" t="inlineStr">
         <is>
-          <t>轮毂电机 +2.48%</t>
+          <t>轮毂电机 +2.43%</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
@@ -2430,7 +2430,7 @@
         </is>
       </c>
       <c r="E9" s="19" t="n">
-        <v>2.48</v>
+        <v>2.43</v>
       </c>
       <c r="F9" s="23" t="inlineStr">
         <is>
@@ -2470,10 +2470,10 @@
         <v>10.51</v>
       </c>
       <c r="O9" s="19" t="n">
-        <v>6.81</v>
+        <v>6.79</v>
       </c>
       <c r="P9" s="19" t="n">
-        <v>3.44</v>
+        <v>3.43</v>
       </c>
       <c r="Q9" s="19" t="n">
         <v>1.34</v>
@@ -2486,14 +2486,14 @@
       </c>
       <c r="T9" s="12" t="inlineStr">
         <is>
-          <t>轮毂电机 +2.48%</t>
+          <t>轮毂电机 +2.43%</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
@@ -2510,7 +2510,7 @@
         </is>
       </c>
       <c r="E10" s="24" t="n">
-        <v>1.05</v>
+        <v>0.99</v>
       </c>
       <c r="F10" s="20" t="inlineStr">
         <is>
@@ -2550,7 +2550,7 @@
         <v>10.64</v>
       </c>
       <c r="O10" s="24" t="n">
-        <v>1.56</v>
+        <v>1.57</v>
       </c>
       <c r="P10" s="24" t="n">
         <v>1.26</v>
@@ -2566,14 +2566,14 @@
       </c>
       <c r="T10" s="15" t="inlineStr">
         <is>
-          <t>退税商店 +1.05%</t>
+          <t>退税商店 +0.99%</t>
         </is>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
@@ -2590,7 +2590,7 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>1.05</v>
+        <v>0.99</v>
       </c>
       <c r="F11" s="20" t="inlineStr">
         <is>
@@ -2630,10 +2630,10 @@
         <v>12.33</v>
       </c>
       <c r="O11" s="24" t="n">
-        <v>5.19</v>
+        <v>5.12</v>
       </c>
       <c r="P11" s="24" t="n">
-        <v>3.31</v>
+        <v>3.27</v>
       </c>
       <c r="Q11" s="24" t="n">
         <v>1.46</v>
@@ -2646,14 +2646,14 @@
       </c>
       <c r="T11" s="15" t="inlineStr">
         <is>
-          <t>退税商店 +1.05%</t>
+          <t>退税商店 +0.99%</t>
         </is>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
@@ -2670,7 +2670,7 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>1.05</v>
+        <v>0.99</v>
       </c>
       <c r="F12" s="20" t="inlineStr">
         <is>
@@ -2726,14 +2726,14 @@
       </c>
       <c r="T12" s="15" t="inlineStr">
         <is>
-          <t>退税商店 +1.05%</t>
+          <t>退税商店 +0.99%</t>
         </is>
       </c>
     </row>
     <row r="13" ht="38" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
@@ -2750,7 +2750,7 @@
         </is>
       </c>
       <c r="E13" s="19" t="n">
-        <v>0.27</v>
+        <v>0.13</v>
       </c>
       <c r="F13" s="20" t="inlineStr">
         <is>
@@ -2781,39 +2781,39 @@
         </is>
       </c>
       <c r="L13" s="19" t="n">
-        <v>11.94</v>
+        <v>11.92</v>
       </c>
       <c r="M13" s="22" t="n">
-        <v>5.57</v>
+        <v>5.39</v>
       </c>
       <c r="N13" s="22" t="n">
-        <v>4.01</v>
+        <v>3.83</v>
       </c>
       <c r="O13" s="19" t="n">
-        <v>2.42</v>
+        <v>2.48</v>
       </c>
       <c r="P13" s="19" t="n">
-        <v>2.14</v>
+        <v>2.18</v>
       </c>
       <c r="Q13" s="19" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
       <c r="R13" s="19" t="n">
-        <v>-40.54</v>
+        <v>-40.64</v>
       </c>
       <c r="S13" s="19" t="n">
-        <v>15.14</v>
+        <v>14.95</v>
       </c>
       <c r="T13" s="12" t="inlineStr">
         <is>
-          <t>大盘价值 +0.27%</t>
+          <t>大盘价值 +0.13%</t>
         </is>
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B14" s="12" t="inlineStr">
@@ -2830,7 +2830,7 @@
         </is>
       </c>
       <c r="E14" s="19" t="n">
-        <v>0.27</v>
+        <v>0.13</v>
       </c>
       <c r="F14" s="20" t="inlineStr">
         <is>
@@ -2842,58 +2842,58 @@
       </c>
       <c r="H14" s="21" t="inlineStr">
         <is>
-          <t>601825</t>
+          <t>002379</t>
         </is>
       </c>
       <c r="I14" s="12" t="inlineStr">
         <is>
-          <t>沪农商行</t>
+          <t>宏桥控股</t>
         </is>
       </c>
       <c r="J14" s="12" t="inlineStr">
         <is>
-          <t>银行Ⅱ</t>
+          <t>工业金属</t>
         </is>
       </c>
       <c r="K14" s="12" t="inlineStr">
         <is>
-          <t>低市净率、大盘价值</t>
+          <t>大盘价值、股权集中</t>
         </is>
       </c>
       <c r="L14" s="19" t="n">
-        <v>9.19</v>
+        <v>14.55</v>
       </c>
       <c r="M14" s="22" t="n">
-        <v>4.91</v>
+        <v>4.45</v>
       </c>
       <c r="N14" s="22" t="n">
-        <v>6.37</v>
+        <v>1.75</v>
       </c>
       <c r="O14" s="19" t="n">
-        <v>0.5600000000000001</v>
+        <v>3.53</v>
       </c>
       <c r="P14" s="19" t="n">
-        <v>1.95</v>
+        <v>1.47</v>
       </c>
       <c r="Q14" s="19" t="n">
-        <v>1.16</v>
+        <v>0.99</v>
       </c>
       <c r="R14" s="19" t="n">
-        <v>0</v>
+        <v>-54.93</v>
       </c>
       <c r="S14" s="19" t="n">
-        <v>26.93</v>
+        <v>6.05</v>
       </c>
       <c r="T14" s="12" t="inlineStr">
         <is>
-          <t>大盘价值 +0.27%</t>
+          <t>大盘价值 +0.13%</t>
         </is>
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -2910,7 +2910,7 @@
         </is>
       </c>
       <c r="E15" s="19" t="n">
-        <v>0.27</v>
+        <v>0.13</v>
       </c>
       <c r="F15" s="20" t="inlineStr">
         <is>
@@ -2922,58 +2922,58 @@
       </c>
       <c r="H15" s="21" t="inlineStr">
         <is>
-          <t>002379</t>
+          <t>000708</t>
         </is>
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>宏桥控股</t>
+          <t>中信特钢</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
         <is>
-          <t>工业金属</t>
+          <t>特钢Ⅱ</t>
         </is>
       </c>
       <c r="K15" s="12" t="inlineStr">
         <is>
-          <t>大盘价值、股权集中</t>
+          <t>地下管网、大盘价值、社保新进、股权集中、行业龙头</t>
         </is>
       </c>
       <c r="L15" s="19" t="n">
-        <v>14.6</v>
+        <v>12.09</v>
       </c>
       <c r="M15" s="22" t="n">
-        <v>4.81</v>
-      </c>
-      <c r="N15" s="22" t="n">
-        <v>2.1</v>
+        <v>4.4</v>
+      </c>
+      <c r="N15" s="27" t="n">
+        <v>-8.48</v>
       </c>
       <c r="O15" s="19" t="n">
-        <v>3.51</v>
+        <v>0.62</v>
       </c>
       <c r="P15" s="19" t="n">
-        <v>1.46</v>
+        <v>2.15</v>
       </c>
       <c r="Q15" s="19" t="n">
-        <v>0.99</v>
+        <v>1.61</v>
       </c>
       <c r="R15" s="19" t="n">
-        <v>-54.77</v>
+        <v>-30.44</v>
       </c>
       <c r="S15" s="19" t="n">
-        <v>6.41</v>
+        <v>4.4</v>
       </c>
       <c r="T15" s="12" t="inlineStr">
         <is>
-          <t>大盘价值 +0.27%</t>
+          <t>大盘价值 +0.13%</t>
         </is>
       </c>
     </row>
     <row r="16" ht="38" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="E16" s="19" t="n">
-        <v>-0.15</v>
+        <v>-0.26</v>
       </c>
       <c r="F16" s="20" t="inlineStr">
         <is>
@@ -3030,10 +3030,10 @@
         <v>12.33</v>
       </c>
       <c r="O16" s="19" t="n">
-        <v>5.19</v>
+        <v>5.12</v>
       </c>
       <c r="P16" s="19" t="n">
-        <v>3.31</v>
+        <v>3.27</v>
       </c>
       <c r="Q16" s="19" t="n">
         <v>1.46</v>
@@ -3046,14 +3046,14 @@
       </c>
       <c r="T16" s="12" t="inlineStr">
         <is>
-          <t>免税概念 -0.15%</t>
+          <t>免税概念 -0.26%</t>
         </is>
       </c>
     </row>
     <row r="17" ht="38" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -3070,7 +3070,7 @@
         </is>
       </c>
       <c r="E17" s="19" t="n">
-        <v>-0.15</v>
+        <v>-0.26</v>
       </c>
       <c r="F17" s="20" t="inlineStr">
         <is>
@@ -3082,58 +3082,58 @@
       </c>
       <c r="H17" s="21" t="inlineStr">
         <is>
-          <t>600029</t>
+          <t>600694</t>
         </is>
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
-          <t>南方航空</t>
+          <t>大商股份</t>
         </is>
       </c>
       <c r="J17" s="12" t="inlineStr">
         <is>
-          <t>航空机场</t>
+          <t>一般零售</t>
         </is>
       </c>
       <c r="K17" s="12" t="inlineStr">
         <is>
-          <t>免税概念、大盘成长、零售概念</t>
+          <t>东北振兴、低市净率、免税概念、内贸流通、社保新进、零售概念</t>
         </is>
       </c>
       <c r="L17" s="19" t="n">
-        <v>4.81</v>
+        <v>15.15</v>
       </c>
       <c r="M17" s="22" t="n">
-        <v>0.84</v>
+        <v>0.73</v>
       </c>
       <c r="N17" s="22" t="n">
-        <v>2.78</v>
+        <v>3.84</v>
       </c>
       <c r="O17" s="19" t="n">
-        <v>0.42</v>
+        <v>1.51</v>
       </c>
       <c r="P17" s="19" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="Q17" s="19" t="n">
         <v>1.32</v>
       </c>
-      <c r="Q17" s="19" t="n">
-        <v>1.17</v>
-      </c>
       <c r="R17" s="19" t="n">
-        <v>-41.98</v>
+        <v>-12.53</v>
       </c>
       <c r="S17" s="19" t="n">
-        <v>3</v>
+        <v>14.51</v>
       </c>
       <c r="T17" s="12" t="inlineStr">
         <is>
-          <t>免税概念 -0.15%</t>
+          <t>免税概念 -0.26%</t>
         </is>
       </c>
     </row>
     <row r="18" ht="38" customHeight="1">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
@@ -3150,7 +3150,7 @@
         </is>
       </c>
       <c r="E18" s="19" t="n">
-        <v>-0.15</v>
+        <v>-0.26</v>
       </c>
       <c r="F18" s="20" t="inlineStr">
         <is>
@@ -3162,58 +3162,58 @@
       </c>
       <c r="H18" s="21" t="inlineStr">
         <is>
-          <t>600694</t>
+          <t>600029</t>
         </is>
       </c>
       <c r="I18" s="12" t="inlineStr">
         <is>
-          <t>大商股份</t>
+          <t>南方航空</t>
         </is>
       </c>
       <c r="J18" s="12" t="inlineStr">
         <is>
-          <t>一般零售</t>
+          <t>航空机场</t>
         </is>
       </c>
       <c r="K18" s="12" t="inlineStr">
         <is>
-          <t>东北振兴、低市净率、免税概念、内贸流通、社保新进、零售概念</t>
+          <t>免税概念、大盘成长、零售概念</t>
         </is>
       </c>
       <c r="L18" s="19" t="n">
-        <v>15.16</v>
+        <v>4.8</v>
       </c>
       <c r="M18" s="22" t="n">
-        <v>0.8</v>
+        <v>0.63</v>
       </c>
       <c r="N18" s="22" t="n">
-        <v>3.91</v>
+        <v>2.56</v>
       </c>
       <c r="O18" s="19" t="n">
-        <v>1.44</v>
+        <v>0.43</v>
       </c>
       <c r="P18" s="19" t="n">
-        <v>1.59</v>
+        <v>1.33</v>
       </c>
       <c r="Q18" s="19" t="n">
-        <v>1.31</v>
+        <v>1.17</v>
       </c>
       <c r="R18" s="19" t="n">
-        <v>-12.47</v>
+        <v>-42.1</v>
       </c>
       <c r="S18" s="19" t="n">
-        <v>14.59</v>
+        <v>2.78</v>
       </c>
       <c r="T18" s="12" t="inlineStr">
         <is>
-          <t>免税概念 -0.15%</t>
+          <t>免税概念 -0.26%</t>
         </is>
       </c>
     </row>
     <row r="19" ht="38" customHeight="1">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -3230,7 +3230,7 @@
         </is>
       </c>
       <c r="E19" s="19" t="n">
-        <v>-0.39</v>
+        <v>-0.47</v>
       </c>
       <c r="F19" s="20" t="inlineStr">
         <is>
@@ -3270,10 +3270,10 @@
         <v>8.359999999999999</v>
       </c>
       <c r="O19" s="19" t="n">
-        <v>12.18</v>
+        <v>12.08</v>
       </c>
       <c r="P19" s="19" t="n">
-        <v>1.43</v>
+        <v>1.42</v>
       </c>
       <c r="Q19" s="19" t="n">
         <v>1.27</v>
@@ -3286,14 +3286,14 @@
       </c>
       <c r="T19" s="12" t="inlineStr">
         <is>
-          <t>汽车整车 -0.39%</t>
+          <t>汽车整车 -0.47%</t>
         </is>
       </c>
     </row>
     <row r="20" ht="38" customHeight="1">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B20" s="12" t="inlineStr">
@@ -3310,7 +3310,7 @@
         </is>
       </c>
       <c r="E20" s="19" t="n">
-        <v>-0.39</v>
+        <v>-0.47</v>
       </c>
       <c r="F20" s="20" t="inlineStr">
         <is>
@@ -3341,39 +3341,39 @@
         </is>
       </c>
       <c r="L20" s="19" t="n">
-        <v>20.8</v>
+        <v>20.84</v>
       </c>
       <c r="M20" s="22" t="n">
-        <v>2.06</v>
+        <v>2.26</v>
       </c>
       <c r="N20" s="22" t="n">
-        <v>2.72</v>
+        <v>2.91</v>
       </c>
       <c r="O20" s="19" t="n">
-        <v>0.79</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="P20" s="19" t="n">
-        <v>1.15</v>
+        <v>1.17</v>
       </c>
       <c r="Q20" s="19" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="R20" s="19" t="n">
-        <v>-19.75</v>
+        <v>-19.6</v>
       </c>
       <c r="S20" s="19" t="n">
-        <v>31.4</v>
+        <v>31.65</v>
       </c>
       <c r="T20" s="12" t="inlineStr">
         <is>
-          <t>汽车整车 -0.39%</t>
+          <t>汽车整车 -0.47%</t>
         </is>
       </c>
     </row>
     <row r="21" ht="38" customHeight="1">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>10-27午盘</t>
+          <t>10-27收盘</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
@@ -3390,7 +3390,7 @@
         </is>
       </c>
       <c r="E21" s="19" t="n">
-        <v>-0.39</v>
+        <v>-0.47</v>
       </c>
       <c r="F21" s="20" t="inlineStr">
         <is>
@@ -3430,10 +3430,10 @@
         <v>0.28</v>
       </c>
       <c r="O21" s="19" t="n">
-        <v>0.6</v>
+        <v>0.62</v>
       </c>
       <c r="P21" s="19" t="n">
-        <v>0.58</v>
+        <v>0.59</v>
       </c>
       <c r="Q21" s="19" t="n">
         <v>0.8100000000000001</v>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="T21" s="12" t="inlineStr">
         <is>
-          <t>汽车整车 -0.39%</t>
+          <t>汽车整车 -0.47%</t>
         </is>
       </c>
     </row>

</xml_diff>